<commit_message>
Add MS Teams integration feature
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,68 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+        <bgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF1DE"/>
+        <bgColor rgb="00EBF1DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+        <bgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +94,47 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,116 +500,1014 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Workload</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Manager_Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>alice@demo.com</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>SAP_Support</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Kumar</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>kumar@demo.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Bob</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>bob@demo.com</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>SAP_Support</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Kumar</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>kumar@demo.com</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Charlie</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>charlie@demo.com</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Database_Admin</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Ms. Sharma</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>sharma@demo.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>david@demo.com</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Network_Ops</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Low</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Mr. Patel</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>patel@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Eve</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>eve@demo.com</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Network_Ops</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Mr. Patel</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>patel@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Frank</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>frank@demo.com</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Network_Ops</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Mr. Patel</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>patel@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>grace@demo.com</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Database_Admin</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Ms. Sharma</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>sharma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Henry</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>henry@demo.com</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Database_Admin</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Ms. Sharma</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>sharma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>irene@demo.com</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>SAP_Support</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Kumar</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>kumar@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Jack</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>jack@demo.com</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>SAP_Support</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Kumar</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>kumar@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Karen</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>karen@demo.com</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Software_Support</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Ms. Nair</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>nair@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Leo</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>leo@demo.com</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Software_Support</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Ms. Nair</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>nair@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Mia</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>mia@demo.com</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Software_Support</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Ms. Nair</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>nair@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Nathan</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>nathan@demo.com</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Software_Support</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Ms. Nair</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>nair@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Olivia</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>olivia@demo.com</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Software_Support</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Ms. Nair</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>nair@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>paul@demo.com</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Hardware_Support</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Mr. Verma</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>verma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Quinn</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>quinn@demo.com</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Hardware_Support</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Mr. Verma</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>verma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Rachel</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>rachel@demo.com</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Hardware_Support</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Mr. Verma</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>verma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>sam@demo.com</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Hardware_Support</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Mr. Verma</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>verma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Tina</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>tina@demo.com</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Hardware_Support</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Mr. Verma</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>verma@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Uma</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>uma@demo.com</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Cloud_Ops</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Mr. Reddy</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>reddy@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Victor</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>victor@demo.com</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Cloud_Ops</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Mr. Reddy</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>reddy@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Wendy</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>wendy@demo.com</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Cloud_Ops</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Mr. Reddy</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>reddy@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Xander</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>xander@demo.com</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Cloud_Ops</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Mr. Reddy</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>reddy@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Yara</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>yara@demo.com</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Cloud_Ops</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Mr. Reddy</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>reddy@demo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Zoe</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>zoe@demo.com</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Cloud_Ops</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Mr. Reddy</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>reddy@demo.com</t>
         </is>
       </c>
     </row>

</xml_diff>